<commit_message>
feat: visualisation final commit
</commit_message>
<xml_diff>
--- a/projects/team_ronin/navjeevan_backend/ds.xlsx
+++ b/projects/team_ronin/navjeevan_backend/ds.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\grizz\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{40DC31AC-4D94-431F-B939-3F8BC76C6758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6077A4E-0720-45B1-80B0-DA84E502A188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -212,9 +212,6 @@
     <t>Siraha</t>
   </si>
   <si>
-    <t>Dhanusha</t>
-  </si>
-  <si>
     <t>Mahottari</t>
   </si>
   <si>
@@ -326,18 +323,9 @@
     <t>Rolpa</t>
   </si>
   <si>
-    <t>Rukum East</t>
-  </si>
-  <si>
-    <t>Kapilvastu</t>
-  </si>
-  <si>
     <t>Rupandehi</t>
   </si>
   <si>
-    <t>Nawalparasi West</t>
-  </si>
-  <si>
     <t>Dang</t>
   </si>
   <si>
@@ -564,6 +552,18 @@
   </si>
   <si>
     <t>9 districts — Far-western Nepal</t>
+  </si>
+  <si>
+    <t>Kapilbastu</t>
+  </si>
+  <si>
+    <t>Rukum</t>
+  </si>
+  <si>
+    <t>Nawalparasi</t>
+  </si>
+  <si>
+    <t>Dhanusa</t>
   </si>
 </sst>
 </file>
@@ -2670,7 +2670,7 @@
         <v>55</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>63</v>
+        <v>180</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>61</v>
@@ -2759,7 +2759,7 @@
         <v>55</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>61</v>
@@ -2848,7 +2848,7 @@
         <v>55</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>61</v>
@@ -2937,7 +2937,7 @@
         <v>55</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>61</v>
@@ -3026,7 +3026,7 @@
         <v>42</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>61</v>
@@ -3115,7 +3115,7 @@
         <v>42</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>61</v>
@@ -3204,10 +3204,10 @@
         <v>42</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>70</v>
       </c>
       <c r="D26" s="4">
         <v>296192</v>
@@ -3293,10 +3293,10 @@
         <v>42</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D27" s="6">
         <v>209491</v>
@@ -3382,10 +3382,10 @@
         <v>42</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D28" s="4">
         <v>186557</v>
@@ -3471,10 +3471,10 @@
         <v>42</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D29" s="6">
         <v>287798</v>
@@ -3560,10 +3560,10 @@
         <v>46</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D30" s="8">
         <v>381937</v>
@@ -3649,10 +3649,10 @@
         <v>46</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D31" s="8">
         <v>709100</v>
@@ -3738,10 +3738,10 @@
         <v>46</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D32" s="8">
         <v>439374</v>
@@ -3827,10 +3827,10 @@
         <v>46</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D33" s="8">
         <v>2000565</v>
@@ -3916,10 +3916,10 @@
         <v>42</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D34" s="4">
         <v>277471</v>
@@ -4005,10 +4005,10 @@
         <v>55</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D35" s="10">
         <v>43300</v>
@@ -4094,10 +4094,10 @@
         <v>42</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D36" s="4">
         <v>336067</v>
@@ -4183,10 +4183,10 @@
         <v>42</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D37" s="6">
         <v>419299</v>
@@ -4272,10 +4272,10 @@
         <v>46</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D38" s="8">
         <v>579250</v>
@@ -4361,10 +4361,10 @@
         <v>42</v>
       </c>
       <c r="B39" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C39" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>84</v>
       </c>
       <c r="D39" s="6">
         <v>258474</v>
@@ -4450,10 +4450,10 @@
         <v>42</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D40" s="4">
         <v>167724</v>
@@ -4539,10 +4539,10 @@
         <v>42</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D41" s="6">
         <v>323288</v>
@@ -4628,10 +4628,10 @@
         <v>42</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D42" s="4">
         <v>289148</v>
@@ -4717,10 +4717,10 @@
         <v>46</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D43" s="8">
         <v>492098</v>
@@ -4806,10 +4806,10 @@
         <v>55</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D44" s="10">
         <v>6538</v>
@@ -4895,10 +4895,10 @@
         <v>55</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D45" s="10">
         <v>13452</v>
@@ -4984,10 +4984,10 @@
         <v>55</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D46" s="10">
         <v>115285</v>
@@ -5073,10 +5073,10 @@
         <v>42</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D47" s="6">
         <v>146590</v>
@@ -5162,10 +5162,10 @@
         <v>42</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D48" s="4">
         <v>268613</v>
@@ -5251,10 +5251,10 @@
         <v>42</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D49" s="6">
         <v>344400</v>
@@ -5340,10 +5340,10 @@
         <v>42</v>
       </c>
       <c r="B50" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C50" s="5" t="s">
         <v>95</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>96</v>
       </c>
       <c r="D50" s="4">
         <v>268613</v>
@@ -5429,10 +5429,10 @@
         <v>42</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D51" s="6">
         <v>197632</v>
@@ -5518,10 +5518,10 @@
         <v>42</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D52" s="4">
         <v>281945</v>
@@ -5607,10 +5607,10 @@
         <v>55</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D53" s="10">
         <v>213683</v>
@@ -5696,10 +5696,10 @@
         <v>55</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D54" s="10">
         <v>224506</v>
@@ -5785,10 +5785,10 @@
         <v>55</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>101</v>
+        <v>178</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D55" s="10">
         <v>54154</v>
@@ -5874,10 +5874,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>102</v>
+        <v>177</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D56" s="10">
         <v>672578</v>
@@ -5963,10 +5963,10 @@
         <v>46</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D57" s="8">
         <v>880196</v>
@@ -6052,10 +6052,10 @@
         <v>42</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>104</v>
+        <v>179</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D58" s="4">
         <v>390000</v>
@@ -6141,10 +6141,10 @@
         <v>42</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D59" s="6">
         <v>551097</v>
@@ -6230,10 +6230,10 @@
         <v>42</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D60" s="4">
         <v>491313</v>
@@ -6319,10 +6319,10 @@
         <v>42</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D61" s="6">
         <v>426576</v>
@@ -6408,10 +6408,10 @@
         <v>55</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D62" s="10">
         <v>36700</v>
@@ -6497,10 +6497,10 @@
         <v>55</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D63" s="10">
         <v>55286</v>
@@ -6586,10 +6586,10 @@
         <v>55</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D64" s="10">
         <v>50858</v>
@@ -6675,10 +6675,10 @@
         <v>55</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D65" s="10">
         <v>108921</v>
@@ -6764,10 +6764,10 @@
         <v>55</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D66" s="10">
         <v>136948</v>
@@ -6853,10 +6853,10 @@
         <v>55</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D67" s="10">
         <v>171304</v>
@@ -6942,10 +6942,10 @@
         <v>55</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D68" s="10">
         <v>156984</v>
@@ -7031,10 +7031,10 @@
         <v>55</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D69" s="10">
         <v>242444</v>
@@ -7120,10 +7120,10 @@
         <v>42</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D70" s="4">
         <v>350804</v>
@@ -7209,10 +7209,10 @@
         <v>55</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D71" s="10">
         <v>261770</v>
@@ -7298,10 +7298,10 @@
         <v>55</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D72" s="10">
         <v>134912</v>
@@ -7387,10 +7387,10 @@
         <v>55</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D73" s="10">
         <v>195159</v>
@@ -7476,10 +7476,10 @@
         <v>55</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D74" s="10">
         <v>261462</v>
@@ -7565,10 +7565,10 @@
         <v>55</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D75" s="10">
         <v>207082</v>
@@ -7654,10 +7654,10 @@
         <v>42</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D76" s="4">
         <v>143246</v>
@@ -7743,10 +7743,10 @@
         <v>55</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D77" s="10">
         <v>283459</v>
@@ -7832,10 +7832,10 @@
         <v>55</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D78" s="10">
         <v>133274</v>
@@ -7921,10 +7921,10 @@
         <v>42</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D79" s="6">
         <v>451248</v>
@@ -8010,10 +8010,10 @@
         <v>42</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D80" s="4">
         <v>775709</v>
@@ -8114,16 +8114,16 @@
   <sheetData>
     <row r="1" spans="1:2" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B1" s="18"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -8131,7 +8131,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -8139,7 +8139,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -8147,7 +8147,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -8155,7 +8155,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -8163,7 +8163,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -8171,7 +8171,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -8179,47 +8179,47 @@
         <v>8</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="12" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="12" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -8227,7 +8227,7 @@
         <v>25</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -8235,7 +8235,7 @@
         <v>26</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
@@ -8243,7 +8243,7 @@
         <v>27</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
@@ -8251,7 +8251,7 @@
         <v>28</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
@@ -8259,7 +8259,7 @@
         <v>29</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
@@ -8267,7 +8267,7 @@
         <v>30</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
@@ -8275,7 +8275,7 @@
         <v>31</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
@@ -8283,15 +8283,15 @@
         <v>32</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="12" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
@@ -8299,7 +8299,7 @@
         <v>35</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
@@ -8307,7 +8307,7 @@
         <v>36</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
@@ -8315,7 +8315,7 @@
         <v>37</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
@@ -8323,7 +8323,7 @@
         <v>38</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
@@ -8331,7 +8331,7 @@
         <v>39</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
@@ -8339,7 +8339,7 @@
         <v>40</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
@@ -8347,42 +8347,42 @@
         <v>41</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B33" s="11"/>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="14" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="15" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="16" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" s="11" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B38" s="11"/>
     </row>
@@ -8391,7 +8391,7 @@
         <v>44</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
@@ -8399,47 +8399,47 @@
         <v>61</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" s="12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" s="12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" s="12" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" s="12" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>